<commit_message>
all code for the draft
</commit_message>
<xml_diff>
--- a/Datasets/Riskperceptiondataset_201125.xlsx
+++ b/Datasets/Riskperceptiondataset_201125.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3ca3652908a58f1c/BEP/BranchInes/Datasets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/idattatreya_tudelft_nl/Documents/BEP/BranchInes/Datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23BA4258-C1F5-494F-94D9-488904206FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{23BA4258-C1F5-494F-94D9-488904206FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{669F39C9-699E-4637-98FA-557A77438F0E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="18426" windowHeight="11746" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AllsurveyforLCA" sheetId="3" r:id="rId1"/>
@@ -569,7 +569,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss\ \U\T\C"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -632,7 +632,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -645,6 +645,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -935,14 +939,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{043D802E-6803-430C-9369-26993460540E}">
   <dimension ref="A1:X160"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.7109375" customWidth="1"/>
+    <col min="1" max="1" width="13.703125" customWidth="1"/>
+    <col min="2" max="2" width="10.703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.703125" customWidth="1"/>
+    <col min="23" max="23" width="14.41015625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1016,7 +1021,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1087,7 +1092,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1158,7 +1163,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1229,7 +1234,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1300,7 +1305,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:24">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1371,7 +1376,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1442,7 +1447,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1513,7 +1518,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:24">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1584,7 +1589,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1655,7 +1660,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:24">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1726,7 +1731,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1797,7 +1802,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1868,7 +1873,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1939,7 +1944,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2010,7 +2015,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.5">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2081,7 +2086,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:23">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2152,7 +2157,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:23">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2223,7 +2228,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:23">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2294,7 +2299,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:23">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2365,7 +2370,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:23">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2436,7 +2441,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:23">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2507,7 +2512,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:23">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2578,7 +2583,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:23">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2649,7 +2654,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:23">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2720,7 +2725,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:23">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2791,7 +2796,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:23">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2862,7 +2867,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:23">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2933,7 +2938,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:23">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3004,7 +3009,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:23">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3075,7 +3080,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="31" spans="1:23">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3146,7 +3151,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:23">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A32">
         <v>31</v>
       </c>
@@ -3217,7 +3222,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:23">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A33">
         <v>32</v>
       </c>
@@ -3288,7 +3293,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:23">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3359,7 +3364,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:23">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3430,7 +3435,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:23">
+    <row r="36" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3501,7 +3506,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:23">
+    <row r="37" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3572,7 +3577,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="38" spans="1:23">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3643,7 +3648,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:23">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3714,7 +3719,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:23">
+    <row r="40" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3785,7 +3790,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="41" spans="1:23">
+    <row r="41" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3856,7 +3861,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:23">
+    <row r="42" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3927,7 +3932,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="43" spans="1:23">
+    <row r="43" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A43">
         <v>42</v>
       </c>
@@ -3998,7 +4003,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:23">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A44">
         <v>43</v>
       </c>
@@ -4069,7 +4074,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:23">
+    <row r="45" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A45">
         <v>44</v>
       </c>
@@ -4140,7 +4145,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="46" spans="1:23">
+    <row r="46" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A46">
         <v>45</v>
       </c>
@@ -4211,7 +4216,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="47" spans="1:23">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A47">
         <v>46</v>
       </c>
@@ -4282,7 +4287,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="48" spans="1:23">
+    <row r="48" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A48">
         <v>47</v>
       </c>
@@ -4353,7 +4358,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="49" spans="1:23">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A49">
         <v>48</v>
       </c>
@@ -4424,7 +4429,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:23">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A50">
         <v>49</v>
       </c>
@@ -4495,7 +4500,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="51" spans="1:23">
+    <row r="51" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A51">
         <v>50</v>
       </c>
@@ -4566,7 +4571,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="52" spans="1:23">
+    <row r="52" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4637,7 +4642,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="53" spans="1:23">
+    <row r="53" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A53">
         <v>52</v>
       </c>
@@ -4708,7 +4713,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="54" spans="1:23">
+    <row r="54" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A54">
         <v>53</v>
       </c>
@@ -4779,7 +4784,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="55" spans="1:23">
+    <row r="55" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A55">
         <v>54</v>
       </c>
@@ -4850,7 +4855,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="56" spans="1:23">
+    <row r="56" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A56">
         <v>55</v>
       </c>
@@ -4921,7 +4926,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="57" spans="1:23">
+    <row r="57" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A57">
         <v>56</v>
       </c>
@@ -4992,7 +4997,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:23">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A58">
         <v>57</v>
       </c>
@@ -5063,7 +5068,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="59" spans="1:23">
+    <row r="59" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A59">
         <v>58</v>
       </c>
@@ -5134,7 +5139,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="60" spans="1:23">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A60">
         <v>59</v>
       </c>
@@ -5205,7 +5210,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="61" spans="1:23">
+    <row r="61" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A61">
         <v>60</v>
       </c>
@@ -5276,7 +5281,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="62" spans="1:23">
+    <row r="62" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A62">
         <v>61</v>
       </c>
@@ -5347,7 +5352,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="63" spans="1:23">
+    <row r="63" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A63">
         <v>62</v>
       </c>
@@ -5418,7 +5423,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="64" spans="1:23">
+    <row r="64" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A64">
         <v>63</v>
       </c>
@@ -5489,7 +5494,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="65" spans="1:23">
+    <row r="65" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A65">
         <v>64</v>
       </c>
@@ -5560,7 +5565,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="66" spans="1:23">
+    <row r="66" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A66">
         <v>65</v>
       </c>
@@ -5631,7 +5636,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="67" spans="1:23">
+    <row r="67" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A67">
         <v>66</v>
       </c>
@@ -5702,7 +5707,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="68" spans="1:23">
+    <row r="68" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A68">
         <v>67</v>
       </c>
@@ -5773,7 +5778,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="69" spans="1:23">
+    <row r="69" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A69">
         <v>68</v>
       </c>
@@ -5844,7 +5849,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="70" spans="1:23">
+    <row r="70" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A70">
         <v>69</v>
       </c>
@@ -5915,7 +5920,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="71" spans="1:23">
+    <row r="71" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A71">
         <v>70</v>
       </c>
@@ -5986,7 +5991,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="72" spans="1:23">
+    <row r="72" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A72">
         <v>71</v>
       </c>
@@ -6057,7 +6062,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="73" spans="1:23">
+    <row r="73" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A73">
         <v>72</v>
       </c>
@@ -6128,7 +6133,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="74" spans="1:23">
+    <row r="74" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A74">
         <v>73</v>
       </c>
@@ -6199,7 +6204,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="75" spans="1:23">
+    <row r="75" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A75">
         <v>74</v>
       </c>
@@ -6270,7 +6275,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="76" spans="1:23">
+    <row r="76" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A76">
         <v>75</v>
       </c>
@@ -6341,7 +6346,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="77" spans="1:23">
+    <row r="77" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A77">
         <v>76</v>
       </c>
@@ -6412,7 +6417,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="78" spans="1:23">
+    <row r="78" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A78">
         <v>77</v>
       </c>
@@ -6483,7 +6488,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="79" spans="1:23">
+    <row r="79" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A79">
         <v>78</v>
       </c>
@@ -6554,7 +6559,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="80" spans="1:23">
+    <row r="80" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A80">
         <f>A79+1</f>
         <v>79</v>
@@ -6626,7 +6631,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="81" spans="1:23">
+    <row r="81" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A81">
         <f>A80+1</f>
         <v>80</v>
@@ -6698,7 +6703,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="82" spans="1:23">
+    <row r="82" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A82">
         <f t="shared" ref="A82:A145" si="0">A81+1</f>
         <v>81</v>
@@ -6770,7 +6775,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="83" spans="1:23">
+    <row r="83" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A83">
         <f t="shared" si="0"/>
         <v>82</v>
@@ -6842,7 +6847,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="84" spans="1:23">
+    <row r="84" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A84">
         <f t="shared" si="0"/>
         <v>83</v>
@@ -6914,7 +6919,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="85" spans="1:23">
+    <row r="85" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A85">
         <f t="shared" si="0"/>
         <v>84</v>
@@ -6986,7 +6991,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="86" spans="1:23">
+    <row r="86" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A86">
         <f t="shared" si="0"/>
         <v>85</v>
@@ -7058,7 +7063,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="87" spans="1:23">
+    <row r="87" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A87">
         <f t="shared" si="0"/>
         <v>86</v>
@@ -7130,7 +7135,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="88" spans="1:23">
+    <row r="88" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A88">
         <f t="shared" si="0"/>
         <v>87</v>
@@ -7202,7 +7207,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="89" spans="1:23">
+    <row r="89" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A89">
         <f t="shared" si="0"/>
         <v>88</v>
@@ -7274,7 +7279,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="90" spans="1:23">
+    <row r="90" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A90">
         <f t="shared" si="0"/>
         <v>89</v>
@@ -7346,7 +7351,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="91" spans="1:23">
+    <row r="91" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A91">
         <f t="shared" si="0"/>
         <v>90</v>
@@ -7418,7 +7423,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="92" spans="1:23">
+    <row r="92" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A92">
         <f t="shared" si="0"/>
         <v>91</v>
@@ -7490,7 +7495,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="93" spans="1:23">
+    <row r="93" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A93">
         <f t="shared" si="0"/>
         <v>92</v>
@@ -7562,7 +7567,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="94" spans="1:23">
+    <row r="94" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A94">
         <f t="shared" si="0"/>
         <v>93</v>
@@ -7634,7 +7639,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="95" spans="1:23">
+    <row r="95" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A95">
         <f t="shared" si="0"/>
         <v>94</v>
@@ -7706,7 +7711,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="96" spans="1:23">
+    <row r="96" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A96">
         <f t="shared" si="0"/>
         <v>95</v>
@@ -7778,7 +7783,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="97" spans="1:23">
+    <row r="97" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A97">
         <f t="shared" si="0"/>
         <v>96</v>
@@ -7850,7 +7855,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="98" spans="1:23">
+    <row r="98" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A98">
         <f t="shared" si="0"/>
         <v>97</v>
@@ -7922,7 +7927,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="99" spans="1:23">
+    <row r="99" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A99">
         <f t="shared" si="0"/>
         <v>98</v>
@@ -7994,7 +7999,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="100" spans="1:23">
+    <row r="100" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A100">
         <f t="shared" si="0"/>
         <v>99</v>
@@ -8066,7 +8071,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="101" spans="1:23">
+    <row r="101" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A101">
         <f t="shared" si="0"/>
         <v>100</v>
@@ -8138,7 +8143,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="102" spans="1:23">
+    <row r="102" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A102">
         <f t="shared" si="0"/>
         <v>101</v>
@@ -8210,7 +8215,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="103" spans="1:23">
+    <row r="103" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A103">
         <f t="shared" si="0"/>
         <v>102</v>
@@ -8282,7 +8287,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="104" spans="1:23">
+    <row r="104" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A104">
         <f t="shared" si="0"/>
         <v>103</v>
@@ -8354,7 +8359,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="105" spans="1:23">
+    <row r="105" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A105">
         <f t="shared" si="0"/>
         <v>104</v>
@@ -8426,7 +8431,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="106" spans="1:23">
+    <row r="106" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A106">
         <f t="shared" si="0"/>
         <v>105</v>
@@ -8441,7 +8446,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="107" spans="1:23">
+    <row r="107" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A107">
         <f t="shared" si="0"/>
         <v>106</v>
@@ -8513,7 +8518,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="108" spans="1:23">
+    <row r="108" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A108">
         <f t="shared" si="0"/>
         <v>107</v>
@@ -8585,7 +8590,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="109" spans="1:23">
+    <row r="109" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A109">
         <f t="shared" si="0"/>
         <v>108</v>
@@ -8657,7 +8662,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="110" spans="1:23">
+    <row r="110" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A110">
         <f t="shared" si="0"/>
         <v>109</v>
@@ -8729,7 +8734,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="111" spans="1:23">
+    <row r="111" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A111">
         <f t="shared" si="0"/>
         <v>110</v>
@@ -8801,7 +8806,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="112" spans="1:23">
+    <row r="112" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A112">
         <f t="shared" si="0"/>
         <v>111</v>
@@ -8873,7 +8878,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="113" spans="1:23">
+    <row r="113" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A113">
         <f t="shared" si="0"/>
         <v>112</v>
@@ -8945,7 +8950,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="114" spans="1:23">
+    <row r="114" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A114">
         <f t="shared" si="0"/>
         <v>113</v>
@@ -9017,7 +9022,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="115" spans="1:23">
+    <row r="115" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A115">
         <f t="shared" si="0"/>
         <v>114</v>
@@ -9089,7 +9094,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="116" spans="1:23">
+    <row r="116" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A116">
         <f t="shared" si="0"/>
         <v>115</v>
@@ -9161,7 +9166,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="117" spans="1:23">
+    <row r="117" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A117">
         <f t="shared" si="0"/>
         <v>116</v>
@@ -9233,7 +9238,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="118" spans="1:23">
+    <row r="118" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A118">
         <f t="shared" si="0"/>
         <v>117</v>
@@ -9305,7 +9310,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="119" spans="1:23">
+    <row r="119" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A119">
         <f t="shared" si="0"/>
         <v>118</v>
@@ -9377,7 +9382,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="120" spans="1:23">
+    <row r="120" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A120">
         <f t="shared" si="0"/>
         <v>119</v>
@@ -9449,7 +9454,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="121" spans="1:23">
+    <row r="121" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A121">
         <f t="shared" si="0"/>
         <v>120</v>
@@ -9521,7 +9526,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="122" spans="1:23">
+    <row r="122" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A122">
         <f t="shared" si="0"/>
         <v>121</v>
@@ -9593,7 +9598,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="123" spans="1:23">
+    <row r="123" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A123">
         <f t="shared" si="0"/>
         <v>122</v>
@@ -9665,7 +9670,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="124" spans="1:23">
+    <row r="124" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A124">
         <f t="shared" si="0"/>
         <v>123</v>
@@ -9737,7 +9742,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="125" spans="1:23">
+    <row r="125" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A125">
         <f t="shared" si="0"/>
         <v>124</v>
@@ -9809,7 +9814,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="126" spans="1:23">
+    <row r="126" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A126">
         <f t="shared" si="0"/>
         <v>125</v>
@@ -9881,7 +9886,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="127" spans="1:23">
+    <row r="127" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A127">
         <f t="shared" si="0"/>
         <v>126</v>
@@ -9953,7 +9958,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="128" spans="1:23">
+    <row r="128" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A128">
         <f t="shared" si="0"/>
         <v>127</v>
@@ -10025,7 +10030,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="129" spans="1:23">
+    <row r="129" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A129">
         <f t="shared" si="0"/>
         <v>128</v>
@@ -10097,7 +10102,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="130" spans="1:23">
+    <row r="130" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A130">
         <f t="shared" si="0"/>
         <v>129</v>
@@ -10169,7 +10174,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="131" spans="1:23">
+    <row r="131" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A131">
         <f t="shared" si="0"/>
         <v>130</v>
@@ -10241,7 +10246,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="132" spans="1:23">
+    <row r="132" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A132">
         <f t="shared" si="0"/>
         <v>131</v>
@@ -10310,7 +10315,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="133" spans="1:23">
+    <row r="133" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A133">
         <f t="shared" si="0"/>
         <v>132</v>
@@ -10382,7 +10387,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="134" spans="1:23">
+    <row r="134" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A134">
         <f t="shared" si="0"/>
         <v>133</v>
@@ -10454,7 +10459,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="135" spans="1:23">
+    <row r="135" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A135">
         <f t="shared" si="0"/>
         <v>134</v>
@@ -10526,7 +10531,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="136" spans="1:23">
+    <row r="136" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A136">
         <f t="shared" si="0"/>
         <v>135</v>
@@ -10598,7 +10603,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="137" spans="1:23">
+    <row r="137" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A137">
         <f t="shared" si="0"/>
         <v>136</v>
@@ -10670,7 +10675,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="138" spans="1:23">
+    <row r="138" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A138">
         <f t="shared" si="0"/>
         <v>137</v>
@@ -10742,7 +10747,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="139" spans="1:23">
+    <row r="139" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A139">
         <f t="shared" si="0"/>
         <v>138</v>
@@ -10814,7 +10819,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="140" spans="1:23">
+    <row r="140" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A140">
         <f t="shared" si="0"/>
         <v>139</v>
@@ -10886,7 +10891,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="141" spans="1:23">
+    <row r="141" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A141">
         <f t="shared" si="0"/>
         <v>140</v>
@@ -10958,7 +10963,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="142" spans="1:23">
+    <row r="142" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A142">
         <f t="shared" si="0"/>
         <v>141</v>
@@ -11030,7 +11035,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="143" spans="1:23">
+    <row r="143" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A143">
         <f t="shared" si="0"/>
         <v>142</v>
@@ -11102,7 +11107,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="144" spans="1:23">
+    <row r="144" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A144">
         <f t="shared" si="0"/>
         <v>143</v>
@@ -11174,7 +11179,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="145" spans="1:23">
+    <row r="145" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A145">
         <f t="shared" si="0"/>
         <v>144</v>
@@ -11246,7 +11251,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="146" spans="1:23">
+    <row r="146" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A146">
         <f t="shared" ref="A146:A154" si="1">A145+1</f>
         <v>145</v>
@@ -11318,7 +11323,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="147" spans="1:23">
+    <row r="147" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A147">
         <f t="shared" si="1"/>
         <v>146</v>
@@ -11390,7 +11395,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="148" spans="1:23">
+    <row r="148" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A148">
         <f t="shared" si="1"/>
         <v>147</v>
@@ -11462,7 +11467,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="149" spans="1:23">
+    <row r="149" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A149">
         <f t="shared" si="1"/>
         <v>148</v>
@@ -11534,7 +11539,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="150" spans="1:23">
+    <row r="150" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A150">
         <f t="shared" si="1"/>
         <v>149</v>
@@ -11606,7 +11611,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="151" spans="1:23">
+    <row r="151" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A151">
         <f t="shared" si="1"/>
         <v>150</v>
@@ -11678,7 +11683,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="152" spans="1:23">
+    <row r="152" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A152">
         <f t="shared" si="1"/>
         <v>151</v>
@@ -11750,7 +11755,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="153" spans="1:23">
+    <row r="153" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A153">
         <f t="shared" si="1"/>
         <v>152</v>
@@ -11822,7 +11827,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="154" spans="1:23">
+    <row r="154" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A154">
         <f t="shared" si="1"/>
         <v>153</v>
@@ -11894,13 +11899,13 @@
         <v>34</v>
       </c>
     </row>
-    <row r="158" spans="1:23">
+    <row r="158" spans="1:23" x14ac:dyDescent="0.5">
       <c r="B158" s="6"/>
     </row>
-    <row r="159" spans="1:23">
+    <row r="159" spans="1:23" x14ac:dyDescent="0.5">
       <c r="B159" s="6"/>
     </row>
-    <row r="160" spans="1:23">
+    <row r="160" spans="1:23" x14ac:dyDescent="0.5">
       <c r="B160" s="6"/>
     </row>
   </sheetData>
@@ -11911,14 +11916,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A41B2068-C3EB-43C3-AEE2-592B866B1B1C}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <cols>
+    <col min="1" max="1" width="16.5859375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.5">
       <c r="B1" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
         <v>167</v>
       </c>
@@ -11926,7 +11934,7 @@
         <v>45559</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
         <v>168</v>
       </c>
@@ -11934,7 +11942,7 @@
         <v>45923</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
         <v>169</v>
       </c>
@@ -11950,15 +11958,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F58E04D-405E-46DC-8E26-3872CFE84DE0}">
   <dimension ref="A1:AA156"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" customWidth="1"/>
-    <col min="22" max="22" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="12.703125" customWidth="1"/>
+    <col min="3" max="3" width="29.29296875" customWidth="1"/>
+    <col min="4" max="4" width="21.29296875" customWidth="1"/>
+    <col min="22" max="22" width="12.29296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -12029,7 +12037,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:23">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -12100,7 +12108,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:23">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A3">
         <v>2</v>
       </c>
@@ -12171,7 +12179,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:23">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A4">
         <v>3</v>
       </c>
@@ -12242,7 +12250,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:23">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -12313,7 +12321,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:23">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A6">
         <v>5</v>
       </c>
@@ -12384,7 +12392,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:23">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A7">
         <v>6</v>
       </c>
@@ -12455,7 +12463,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:23">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A8">
         <v>7</v>
       </c>
@@ -12526,7 +12534,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:23">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A9">
         <v>8</v>
       </c>
@@ -12597,7 +12605,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:23">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A10">
         <v>9</v>
       </c>
@@ -12668,7 +12676,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:23">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A11">
         <v>10</v>
       </c>
@@ -12739,7 +12747,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:23">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A12">
         <v>11</v>
       </c>
@@ -12810,7 +12818,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:23">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A13">
         <v>12</v>
       </c>
@@ -12881,7 +12889,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:23">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A14">
         <v>13</v>
       </c>
@@ -12952,7 +12960,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:23">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A15">
         <v>14</v>
       </c>
@@ -13023,7 +13031,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:23">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A16">
         <v>15</v>
       </c>
@@ -13094,7 +13102,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:23">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A17">
         <v>16</v>
       </c>
@@ -13165,7 +13173,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:23">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A18">
         <v>17</v>
       </c>
@@ -13236,7 +13244,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:23">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A19">
         <v>18</v>
       </c>
@@ -13307,7 +13315,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:23">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A20">
         <v>19</v>
       </c>
@@ -13378,7 +13386,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:23">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A21">
         <v>20</v>
       </c>
@@ -13449,7 +13457,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:23">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A22">
         <v>21</v>
       </c>
@@ -13520,7 +13528,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:23">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A23">
         <v>22</v>
       </c>
@@ -13591,7 +13599,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:23">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A24">
         <v>23</v>
       </c>
@@ -13662,7 +13670,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:23">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A25">
         <v>24</v>
       </c>
@@ -13733,7 +13741,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:23">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A26">
         <v>25</v>
       </c>
@@ -13804,7 +13812,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:23">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A27">
         <v>26</v>
       </c>
@@ -13875,7 +13883,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:23">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A28">
         <v>27</v>
       </c>
@@ -13946,7 +13954,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:23">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A29">
         <v>28</v>
       </c>
@@ -14017,7 +14025,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:23">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A30">
         <v>29</v>
       </c>
@@ -14088,7 +14096,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="31" spans="1:23">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A31">
         <v>30</v>
       </c>
@@ -14159,7 +14167,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:23">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A32">
         <v>31</v>
       </c>
@@ -14230,7 +14238,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:23">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A33">
         <v>32</v>
       </c>
@@ -14301,7 +14309,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:23">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A34">
         <v>33</v>
       </c>
@@ -14372,7 +14380,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:23">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A35">
         <v>34</v>
       </c>
@@ -14443,7 +14451,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:23">
+    <row r="36" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A36">
         <v>35</v>
       </c>
@@ -14514,7 +14522,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:23">
+    <row r="37" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A37">
         <v>36</v>
       </c>
@@ -14585,7 +14593,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="38" spans="1:23">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A38">
         <v>37</v>
       </c>
@@ -14656,7 +14664,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:23">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A39">
         <v>38</v>
       </c>
@@ -14727,7 +14735,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:23">
+    <row r="40" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A40">
         <v>39</v>
       </c>
@@ -14798,7 +14806,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="41" spans="1:23">
+    <row r="41" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A41">
         <v>40</v>
       </c>
@@ -14869,7 +14877,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:23">
+    <row r="42" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A42">
         <v>41</v>
       </c>
@@ -14940,7 +14948,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="43" spans="1:23">
+    <row r="43" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A43">
         <v>42</v>
       </c>
@@ -15011,7 +15019,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:23">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A44">
         <v>43</v>
       </c>
@@ -15082,7 +15090,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:23">
+    <row r="45" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A45">
         <v>44</v>
       </c>
@@ -15153,7 +15161,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="46" spans="1:23">
+    <row r="46" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A46">
         <v>45</v>
       </c>
@@ -15224,7 +15232,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="47" spans="1:23">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A47">
         <v>46</v>
       </c>
@@ -15295,7 +15303,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="48" spans="1:23">
+    <row r="48" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A48">
         <v>47</v>
       </c>
@@ -15366,7 +15374,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="49" spans="1:23">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A49">
         <v>48</v>
       </c>
@@ -15437,7 +15445,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:23">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A50">
         <v>49</v>
       </c>
@@ -15508,7 +15516,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="51" spans="1:23">
+    <row r="51" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A51">
         <v>50</v>
       </c>
@@ -15579,7 +15587,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="52" spans="1:23">
+    <row r="52" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A52">
         <v>51</v>
       </c>
@@ -15650,7 +15658,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="53" spans="1:23">
+    <row r="53" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A53">
         <v>52</v>
       </c>
@@ -15721,7 +15729,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="54" spans="1:23">
+    <row r="54" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A54">
         <v>53</v>
       </c>
@@ -15792,7 +15800,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="55" spans="1:23">
+    <row r="55" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A55">
         <v>54</v>
       </c>
@@ -15863,7 +15871,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="56" spans="1:23">
+    <row r="56" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A56">
         <v>55</v>
       </c>
@@ -15934,7 +15942,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="57" spans="1:23">
+    <row r="57" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A57">
         <v>56</v>
       </c>
@@ -16005,7 +16013,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:23">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A58">
         <v>57</v>
       </c>
@@ -16076,7 +16084,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="59" spans="1:23">
+    <row r="59" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A59">
         <v>58</v>
       </c>
@@ -16147,7 +16155,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="60" spans="1:23">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A60">
         <v>59</v>
       </c>
@@ -16218,7 +16226,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="61" spans="1:23">
+    <row r="61" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A61">
         <v>60</v>
       </c>
@@ -16289,7 +16297,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="62" spans="1:23">
+    <row r="62" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A62">
         <v>61</v>
       </c>
@@ -16360,7 +16368,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="63" spans="1:23">
+    <row r="63" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A63">
         <v>62</v>
       </c>
@@ -16431,7 +16439,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="64" spans="1:23">
+    <row r="64" spans="1:23" x14ac:dyDescent="0.5">
       <c r="A64">
         <v>63</v>
       </c>
@@ -16502,7 +16510,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="65" spans="1:27">
+    <row r="65" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A65">
         <v>64</v>
       </c>
@@ -16573,7 +16581,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="66" spans="1:27">
+    <row r="66" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A66">
         <v>65</v>
       </c>
@@ -16644,7 +16652,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="67" spans="1:27">
+    <row r="67" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A67">
         <v>66</v>
       </c>
@@ -16715,7 +16723,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="68" spans="1:27">
+    <row r="68" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A68">
         <v>67</v>
       </c>
@@ -16786,7 +16794,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="69" spans="1:27">
+    <row r="69" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A69">
         <v>68</v>
       </c>
@@ -16857,7 +16865,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="70" spans="1:27">
+    <row r="70" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A70">
         <v>69</v>
       </c>
@@ -16928,7 +16936,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="71" spans="1:27">
+    <row r="71" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A71">
         <v>70</v>
       </c>
@@ -16999,7 +17007,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="72" spans="1:27">
+    <row r="72" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A72">
         <v>71</v>
       </c>
@@ -17070,7 +17078,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="73" spans="1:27">
+    <row r="73" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A73">
         <v>72</v>
       </c>
@@ -17141,7 +17149,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="74" spans="1:27">
+    <row r="74" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A74">
         <v>73</v>
       </c>
@@ -17212,7 +17220,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="75" spans="1:27">
+    <row r="75" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A75">
         <v>74</v>
       </c>
@@ -17283,7 +17291,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="76" spans="1:27">
+    <row r="76" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A76">
         <v>75</v>
       </c>
@@ -17354,7 +17362,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="77" spans="1:27">
+    <row r="77" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A77">
         <v>76</v>
       </c>
@@ -17425,7 +17433,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="78" spans="1:27">
+    <row r="78" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A78">
         <v>77</v>
       </c>
@@ -17496,7 +17504,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="79" spans="1:27">
+    <row r="79" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A79">
         <v>78</v>
       </c>
@@ -17567,7 +17575,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="80" spans="1:27">
+    <row r="80" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A80" s="1" t="s">
         <v>0</v>
       </c>
@@ -17650,7 +17658,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="81" spans="1:27">
+    <row r="81" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A81">
         <v>1</v>
       </c>
@@ -17733,7 +17741,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="82" spans="1:27">
+    <row r="82" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A82">
         <v>2</v>
       </c>
@@ -17816,7 +17824,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="83" spans="1:27">
+    <row r="83" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A83">
         <v>3</v>
       </c>
@@ -17899,7 +17907,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="84" spans="1:27">
+    <row r="84" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A84">
         <v>4</v>
       </c>
@@ -17982,7 +17990,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="85" spans="1:27">
+    <row r="85" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A85">
         <v>5</v>
       </c>
@@ -18065,7 +18073,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="86" spans="1:27">
+    <row r="86" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A86">
         <v>6</v>
       </c>
@@ -18148,7 +18156,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="87" spans="1:27">
+    <row r="87" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A87">
         <v>7</v>
       </c>
@@ -18231,7 +18239,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="88" spans="1:27">
+    <row r="88" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A88">
         <v>8</v>
       </c>
@@ -18314,7 +18322,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="89" spans="1:27">
+    <row r="89" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A89">
         <v>9</v>
       </c>
@@ -18397,7 +18405,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="90" spans="1:27">
+    <row r="90" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A90">
         <v>10</v>
       </c>
@@ -18480,7 +18488,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="91" spans="1:27">
+    <row r="91" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A91">
         <v>11</v>
       </c>
@@ -18563,7 +18571,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="92" spans="1:27">
+    <row r="92" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A92">
         <v>12</v>
       </c>
@@ -18646,7 +18654,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="93" spans="1:27">
+    <row r="93" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A93">
         <v>13</v>
       </c>
@@ -18729,7 +18737,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="94" spans="1:27">
+    <row r="94" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A94">
         <v>14</v>
       </c>
@@ -18812,7 +18820,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="95" spans="1:27">
+    <row r="95" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A95">
         <v>15</v>
       </c>
@@ -18895,7 +18903,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="96" spans="1:27">
+    <row r="96" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A96">
         <v>16</v>
       </c>
@@ -18978,7 +18986,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="97" spans="1:27">
+    <row r="97" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A97">
         <v>17</v>
       </c>
@@ -19061,7 +19069,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="98" spans="1:27">
+    <row r="98" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A98">
         <v>18</v>
       </c>
@@ -19144,7 +19152,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="99" spans="1:27">
+    <row r="99" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A99">
         <v>19</v>
       </c>
@@ -19227,7 +19235,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="100" spans="1:27">
+    <row r="100" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A100">
         <v>20</v>
       </c>
@@ -19310,7 +19318,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="101" spans="1:27">
+    <row r="101" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A101">
         <v>21</v>
       </c>
@@ -19393,7 +19401,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="102" spans="1:27">
+    <row r="102" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A102">
         <v>22</v>
       </c>
@@ -19476,7 +19484,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="103" spans="1:27">
+    <row r="103" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A103">
         <v>23</v>
       </c>
@@ -19559,7 +19567,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="104" spans="1:27">
+    <row r="104" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A104">
         <v>24</v>
       </c>
@@ -19642,7 +19650,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="105" spans="1:27">
+    <row r="105" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A105">
         <v>25</v>
       </c>
@@ -19725,7 +19733,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="106" spans="1:27">
+    <row r="106" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A106">
         <v>26</v>
       </c>
@@ -19808,7 +19816,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="107" spans="1:27">
+    <row r="107" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A107">
         <v>27</v>
       </c>
@@ -19826,7 +19834,7 @@
       <c r="T107" s="5"/>
       <c r="U107" s="5"/>
     </row>
-    <row r="108" spans="1:27">
+    <row r="108" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A108">
         <v>28</v>
       </c>
@@ -19909,7 +19917,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="109" spans="1:27">
+    <row r="109" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A109">
         <v>29</v>
       </c>
@@ -19992,7 +20000,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="110" spans="1:27">
+    <row r="110" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A110">
         <v>30</v>
       </c>
@@ -20075,7 +20083,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="111" spans="1:27">
+    <row r="111" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A111">
         <v>31</v>
       </c>
@@ -20158,7 +20166,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="112" spans="1:27">
+    <row r="112" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A112">
         <v>32</v>
       </c>
@@ -20241,7 +20249,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="113" spans="1:27">
+    <row r="113" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A113">
         <v>33</v>
       </c>
@@ -20320,7 +20328,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="114" spans="1:27">
+    <row r="114" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A114">
         <v>34</v>
       </c>
@@ -20403,7 +20411,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="115" spans="1:27">
+    <row r="115" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A115">
         <v>35</v>
       </c>
@@ -20486,7 +20494,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="116" spans="1:27">
+    <row r="116" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A116">
         <v>36</v>
       </c>
@@ -20569,7 +20577,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="117" spans="1:27">
+    <row r="117" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A117">
         <v>37</v>
       </c>
@@ -20652,7 +20660,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="118" spans="1:27">
+    <row r="118" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A118">
         <v>38</v>
       </c>
@@ -20735,7 +20743,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="119" spans="1:27">
+    <row r="119" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A119">
         <v>39</v>
       </c>
@@ -20818,7 +20826,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="120" spans="1:27">
+    <row r="120" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A120">
         <v>40</v>
       </c>
@@ -20901,7 +20909,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="121" spans="1:27">
+    <row r="121" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A121">
         <v>41</v>
       </c>
@@ -20984,7 +20992,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="122" spans="1:27">
+    <row r="122" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A122">
         <v>42</v>
       </c>
@@ -21067,7 +21075,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="123" spans="1:27">
+    <row r="123" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A123">
         <v>43</v>
       </c>
@@ -21150,7 +21158,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="124" spans="1:27">
+    <row r="124" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A124">
         <v>44</v>
       </c>
@@ -21233,7 +21241,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="125" spans="1:27">
+    <row r="125" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A125">
         <v>45</v>
       </c>
@@ -21316,7 +21324,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="126" spans="1:27">
+    <row r="126" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A126">
         <v>46</v>
       </c>
@@ -21399,7 +21407,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="127" spans="1:27">
+    <row r="127" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A127">
         <v>47</v>
       </c>
@@ -21482,7 +21490,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="128" spans="1:27">
+    <row r="128" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A128">
         <v>48</v>
       </c>
@@ -21565,7 +21573,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="129" spans="1:27">
+    <row r="129" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A129">
         <v>49</v>
       </c>
@@ -21648,7 +21656,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="130" spans="1:27">
+    <row r="130" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A130">
         <v>50</v>
       </c>
@@ -21731,7 +21739,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="131" spans="1:27">
+    <row r="131" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A131">
         <v>51</v>
       </c>
@@ -21814,7 +21822,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="132" spans="1:27">
+    <row r="132" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A132">
         <v>52</v>
       </c>
@@ -21897,7 +21905,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="133" spans="1:27">
+    <row r="133" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A133" s="1" t="s">
         <v>0</v>
       </c>
@@ -21980,7 +21988,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="134" spans="1:27">
+    <row r="134" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A134">
         <v>1</v>
       </c>
@@ -22060,7 +22068,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="135" spans="1:27">
+    <row r="135" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A135">
         <v>2</v>
       </c>
@@ -22143,7 +22151,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="136" spans="1:27">
+    <row r="136" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A136">
         <v>3</v>
       </c>
@@ -22226,7 +22234,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="137" spans="1:27">
+    <row r="137" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A137">
         <v>4</v>
       </c>
@@ -22309,7 +22317,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="138" spans="1:27">
+    <row r="138" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A138">
         <v>5</v>
       </c>
@@ -22392,7 +22400,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="139" spans="1:27">
+    <row r="139" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A139">
         <v>6</v>
       </c>
@@ -22475,7 +22483,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="140" spans="1:27">
+    <row r="140" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A140">
         <v>7</v>
       </c>
@@ -22558,7 +22566,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="141" spans="1:27">
+    <row r="141" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A141">
         <v>8</v>
       </c>
@@ -22641,7 +22649,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="142" spans="1:27">
+    <row r="142" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A142">
         <v>9</v>
       </c>
@@ -22724,7 +22732,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="143" spans="1:27">
+    <row r="143" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A143">
         <v>10</v>
       </c>
@@ -22807,7 +22815,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="144" spans="1:27">
+    <row r="144" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A144">
         <v>11</v>
       </c>
@@ -22890,7 +22898,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="145" spans="1:27">
+    <row r="145" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A145">
         <v>12</v>
       </c>
@@ -22973,7 +22981,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="146" spans="1:27">
+    <row r="146" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A146">
         <v>13</v>
       </c>
@@ -23056,7 +23064,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="147" spans="1:27">
+    <row r="147" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A147">
         <v>14</v>
       </c>
@@ -23139,7 +23147,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="148" spans="1:27">
+    <row r="148" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A148">
         <v>15</v>
       </c>
@@ -23222,7 +23230,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="149" spans="1:27">
+    <row r="149" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A149">
         <v>16</v>
       </c>
@@ -23305,7 +23313,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="150" spans="1:27">
+    <row r="150" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A150">
         <v>17</v>
       </c>
@@ -23388,7 +23396,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="151" spans="1:27">
+    <row r="151" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A151">
         <v>18</v>
       </c>
@@ -23471,7 +23479,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="152" spans="1:27">
+    <row r="152" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A152">
         <v>19</v>
       </c>
@@ -23554,7 +23562,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="153" spans="1:27">
+    <row r="153" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A153">
         <v>20</v>
       </c>
@@ -23637,7 +23645,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="154" spans="1:27">
+    <row r="154" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A154">
         <v>21</v>
       </c>
@@ -23720,7 +23728,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="155" spans="1:27">
+    <row r="155" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A155">
         <v>22</v>
       </c>
@@ -23803,7 +23811,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="156" spans="1:27">
+    <row r="156" spans="1:27" x14ac:dyDescent="0.5">
       <c r="A156">
         <v>23</v>
       </c>

</xml_diff>